<commit_message>
Created a copy of the dataset that is reduced to only essential features that will be used for analysis. I also created boxplots of continuous numeric features to assess their spread and check for outliers.
</commit_message>
<xml_diff>
--- a/PCOS Dataset.xlsx
+++ b/PCOS Dataset.xlsx
@@ -1,20 +1,23 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="4" rupBuild="29929"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="4" rupBuild="30026"/>
   <workbookPr defaultThemeVersion="124226"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Lily Jayne Baxendale\Documents\Masters\COM7016 Project\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Lily Jayne Baxendale\masters_project\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{156BB4F6-9161-4E87-A9F5-C7011C88F714}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0A72EC73-B8FB-450F-B1D5-3ACFDAEFF2AC}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="1140" yWindow="1140" windowWidth="15600" windowHeight="8170" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="19090" yWindow="-110" windowWidth="17020" windowHeight="10000" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
   </sheets>
+  <definedNames>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">Sheet1!$A$1:$AZ$469</definedName>
+  </definedNames>
   <calcPr calcId="124519"/>
 </workbook>
 </file>
@@ -74649,6 +74652,7 @@
       </c>
     </row>
   </sheetData>
+  <autoFilter ref="A1:AZ469" xr:uid="{00000000-0001-0000-0000-000000000000}"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
</xml_diff>